<commit_message>
added note archive to contract program, added metadata columns, created a metadata object parser
</commit_message>
<xml_diff>
--- a/010-npm_node/2206JPI02S Anna Waters Creek REV 3 Signage.xlsx
+++ b/010-npm_node/2206JPI02S Anna Waters Creek REV 3 Signage.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:J128"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,6 +419,18 @@
       <c r="F1" t="str">
         <v>5</v>
       </c>
+      <c r="G1" t="str">
+        <v>6</v>
+      </c>
+      <c r="H1" t="str">
+        <v>7</v>
+      </c>
+      <c r="I1" t="str">
+        <v>8</v>
+      </c>
+      <c r="J1" t="str">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -439,6 +451,18 @@
       <c r="F2" t="str">
         <v>TOTAL_COST</v>
       </c>
+      <c r="G2" t="str">
+        <v>CLIENT</v>
+      </c>
+      <c r="H2" t="str">
+        <v>CONTACT</v>
+      </c>
+      <c r="I2" t="str">
+        <v>CONTRACT_NUMBER</v>
+      </c>
+      <c r="J2" t="str">
+        <v>REVISIONS</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -459,6 +483,18 @@
       <c r="F3">
         <v>7800</v>
       </c>
+      <c r="G3" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H3" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J3" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -479,6 +515,18 @@
       <c r="F4">
         <v>4400</v>
       </c>
+      <c r="G4" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H4" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J4" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -499,6 +547,18 @@
       <c r="F5">
         <v>3400</v>
       </c>
+      <c r="G5" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H5" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J5" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -519,6 +579,18 @@
       <c r="F6">
         <v>385</v>
       </c>
+      <c r="G6" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H6" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J6" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -539,6 +611,18 @@
       <c r="F7">
         <v>410</v>
       </c>
+      <c r="G7" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H7" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J7" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -559,6 +643,18 @@
       <c r="F8">
         <v>129</v>
       </c>
+      <c r="G8" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H8" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I8" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J8" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -579,6 +675,18 @@
       <c r="F9">
         <v>89</v>
       </c>
+      <c r="G9" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H9" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I9" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J9" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -599,6 +707,18 @@
       <c r="F10">
         <v>2145</v>
       </c>
+      <c r="G10" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H10" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I10" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J10" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -619,6 +739,18 @@
       <c r="F11">
         <v>1430</v>
       </c>
+      <c r="G11" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H11" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I11" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J11" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -639,6 +771,18 @@
       <c r="F12">
         <v>595</v>
       </c>
+      <c r="G12" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H12" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J12" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -659,6 +803,18 @@
       <c r="F13">
         <v>2970</v>
       </c>
+      <c r="G13" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H13" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I13" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J13" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -679,6 +835,18 @@
       <c r="F14">
         <v>715</v>
       </c>
+      <c r="G14" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H14" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I14" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J14" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -699,6 +867,18 @@
       <c r="F15">
         <v>68</v>
       </c>
+      <c r="G15" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H15" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J15" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -719,6 +899,18 @@
       <c r="F16">
         <v>68</v>
       </c>
+      <c r="G16" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H16" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J16" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -739,6 +931,18 @@
       <c r="F17">
         <v>144</v>
       </c>
+      <c r="G17" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H17" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I17" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J17" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -759,6 +963,18 @@
       <c r="F18">
         <v>136</v>
       </c>
+      <c r="G18" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H18" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I18" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J18" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -779,6 +995,18 @@
       <c r="F19">
         <v>68</v>
       </c>
+      <c r="G19" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H19" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I19" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J19" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -799,6 +1027,18 @@
       <c r="F20">
         <v>156</v>
       </c>
+      <c r="G20" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H20" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I20" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J20" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -819,6 +1059,18 @@
       <c r="F21">
         <v>78</v>
       </c>
+      <c r="G21" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H21" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I21" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J21" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -839,6 +1091,18 @@
       <c r="F22">
         <v>415</v>
       </c>
+      <c r="G22" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H22" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I22" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J22" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -859,6 +1123,18 @@
       <c r="F23">
         <v>98</v>
       </c>
+      <c r="G23" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H23" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I23" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J23" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -879,6 +1155,18 @@
       <c r="F24">
         <v>98</v>
       </c>
+      <c r="G24" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H24" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I24" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J24" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -899,6 +1187,18 @@
       <c r="F25">
         <v>78</v>
       </c>
+      <c r="G25" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H25" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I25" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J25" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -919,6 +1219,18 @@
       <c r="F26">
         <v>415</v>
       </c>
+      <c r="G26" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H26" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I26" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J26" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -939,6 +1251,18 @@
       <c r="F27">
         <v>68</v>
       </c>
+      <c r="G27" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H27" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I27" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J27" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -959,6 +1283,18 @@
       <c r="F28">
         <v>96</v>
       </c>
+      <c r="G28" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H28" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I28" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J28" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -979,6 +1315,18 @@
       <c r="F29">
         <v>48</v>
       </c>
+      <c r="G29" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H29" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I29" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J29" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -999,6 +1347,18 @@
       <c r="F30">
         <v>680</v>
       </c>
+      <c r="G30" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H30" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I30" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J30" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1019,6 +1379,18 @@
       <c r="F31">
         <v>232</v>
       </c>
+      <c r="G31" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H31" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I31" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J31" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1039,6 +1411,18 @@
       <c r="F32">
         <v>7160</v>
       </c>
+      <c r="G32" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H32" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I32" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J32" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1059,6 +1443,18 @@
       <c r="F33">
         <v>4390</v>
       </c>
+      <c r="G33" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H33" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I33" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J33" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1079,6 +1475,18 @@
       <c r="F34">
         <v>9760</v>
       </c>
+      <c r="G34" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H34" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I34" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J34" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1099,6 +1507,18 @@
       <c r="F35">
         <v>1240</v>
       </c>
+      <c r="G35" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H35" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I35" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J35" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1119,6 +1539,18 @@
       <c r="F36">
         <v>555</v>
       </c>
+      <c r="G36" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H36" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I36" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J36" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1139,6 +1571,18 @@
       <c r="F37">
         <v>220</v>
       </c>
+      <c r="G37" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H37" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I37" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J37" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1159,6 +1603,18 @@
       <c r="F38">
         <v>6512</v>
       </c>
+      <c r="G38" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H38" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I38" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J38" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1179,6 +1635,18 @@
       <c r="F39">
         <v>1425</v>
       </c>
+      <c r="G39" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H39" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I39" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J39" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1199,6 +1667,18 @@
       <c r="F40">
         <v>48</v>
       </c>
+      <c r="G40" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H40" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I40" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J40" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1219,6 +1699,18 @@
       <c r="F41">
         <v>624</v>
       </c>
+      <c r="G41" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H41" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I41" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J41" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1239,6 +1731,18 @@
       <c r="F42">
         <v>116</v>
       </c>
+      <c r="G42" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H42" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I42" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J42" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1259,6 +1763,18 @@
       <c r="F43">
         <v>350</v>
       </c>
+      <c r="G43" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H43" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I43" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J43" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1279,6 +1795,18 @@
       <c r="F44">
         <v>245</v>
       </c>
+      <c r="G44" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H44" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I44" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J44" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -1299,6 +1827,18 @@
       <c r="F45">
         <v>240</v>
       </c>
+      <c r="G45" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H45" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I45" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J45" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1319,6 +1859,18 @@
       <c r="F46">
         <v>116</v>
       </c>
+      <c r="G46" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H46" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I46" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J46" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1339,6 +1891,18 @@
       <c r="F47">
         <v>110</v>
       </c>
+      <c r="G47" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H47" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I47" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J47" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1359,6 +1923,18 @@
       <c r="F48">
         <v>1200</v>
       </c>
+      <c r="G48" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H48" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I48" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J48" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1379,6 +1955,18 @@
       <c r="F49">
         <v>110</v>
       </c>
+      <c r="G49" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H49" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I49" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J49" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1399,6 +1987,18 @@
       <c r="F50">
         <v>144</v>
       </c>
+      <c r="G50" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H50" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I50" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J50" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -1419,6 +2019,18 @@
       <c r="F51">
         <v>495</v>
       </c>
+      <c r="G51" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H51" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I51" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J51" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -1439,6 +2051,18 @@
       <c r="F52">
         <v>210</v>
       </c>
+      <c r="G52" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H52" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I52" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J52" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -1459,6 +2083,18 @@
       <c r="F53">
         <v>48</v>
       </c>
+      <c r="G53" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H53" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I53" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J53" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -1479,6 +2115,18 @@
       <c r="F54">
         <v>48</v>
       </c>
+      <c r="G54" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H54" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I54" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J54" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -1499,6 +2147,18 @@
       <c r="F55">
         <v>116</v>
       </c>
+      <c r="G55" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H55" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I55" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J55" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -1519,6 +2179,18 @@
       <c r="F56">
         <v>88</v>
       </c>
+      <c r="G56" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H56" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I56" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J56" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -1539,6 +2211,18 @@
       <c r="F57">
         <v>110</v>
       </c>
+      <c r="G57" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H57" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I57" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J57" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -1559,6 +2243,18 @@
       <c r="F58">
         <v>1488</v>
       </c>
+      <c r="G58" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H58" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I58" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J58" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -1579,6 +2275,18 @@
       <c r="F59">
         <v>110</v>
       </c>
+      <c r="G59" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H59" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I59" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J59" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -1599,6 +2307,18 @@
       <c r="F60">
         <v>144</v>
       </c>
+      <c r="G60" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H60" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I60" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J60" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -1619,6 +2339,18 @@
       <c r="F61">
         <v>495</v>
       </c>
+      <c r="G61" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H61" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I61" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J61" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -1639,6 +2371,18 @@
       <c r="F62">
         <v>210</v>
       </c>
+      <c r="G62" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H62" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I62" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J62" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -1659,6 +2403,18 @@
       <c r="F63">
         <v>48</v>
       </c>
+      <c r="G63" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H63" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I63" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J63" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -1679,6 +2435,18 @@
       <c r="F64">
         <v>144</v>
       </c>
+      <c r="G64" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H64" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I64" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J64" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -1699,6 +2467,18 @@
       <c r="F65">
         <v>116</v>
       </c>
+      <c r="G65" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H65" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I65" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J65" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -1719,6 +2499,18 @@
       <c r="F66">
         <v>1488</v>
       </c>
+      <c r="G66" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H66" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I66" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J66" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -1739,6 +2531,18 @@
       <c r="F67">
         <v>144</v>
       </c>
+      <c r="G67" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H67" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I67" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J67" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -1759,6 +2563,18 @@
       <c r="F68">
         <v>495</v>
       </c>
+      <c r="G68" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H68" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I68" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J68" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -1779,6 +2595,18 @@
       <c r="F69">
         <v>210</v>
       </c>
+      <c r="G69" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H69" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I69" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J69" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -1799,6 +2627,18 @@
       <c r="F70">
         <v>110</v>
       </c>
+      <c r="G70" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H70" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I70" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J70" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -1819,6 +2659,18 @@
       <c r="F71">
         <v>96</v>
       </c>
+      <c r="G71" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H71" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I71" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J71" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -1839,6 +2691,18 @@
       <c r="F72">
         <v>96</v>
       </c>
+      <c r="G72" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H72" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I72" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J72" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -1859,6 +2723,18 @@
       <c r="F73">
         <v>116</v>
       </c>
+      <c r="G73" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H73" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I73" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J73" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -1879,6 +2755,18 @@
       <c r="F74">
         <v>864</v>
       </c>
+      <c r="G74" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H74" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I74" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J74" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -1899,6 +2787,18 @@
       <c r="F75">
         <v>96</v>
       </c>
+      <c r="G75" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H75" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I75" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J75" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -1919,6 +2819,18 @@
       <c r="F76">
         <v>330</v>
       </c>
+      <c r="G76" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H76" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I76" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J76" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -1939,6 +2851,18 @@
       <c r="F77">
         <v>210</v>
       </c>
+      <c r="G77" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H77" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I77" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J77" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -1959,6 +2883,18 @@
       <c r="F78">
         <v>48</v>
       </c>
+      <c r="G78" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H78" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I78" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J78" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -1979,6 +2915,18 @@
       <c r="F79">
         <v>48</v>
       </c>
+      <c r="G79" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H79" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I79" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J79" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -1999,6 +2947,18 @@
       <c r="F80">
         <v>1140</v>
       </c>
+      <c r="G80" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H80" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I80" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J80" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -2019,6 +2979,18 @@
       <c r="F81">
         <v>912</v>
       </c>
+      <c r="G81" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H81" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I81" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J81" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -2039,6 +3011,18 @@
       <c r="F82">
         <v>78</v>
       </c>
+      <c r="G82" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H82" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I82" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J82" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -2059,6 +3043,18 @@
       <c r="F83">
         <v>96</v>
       </c>
+      <c r="G83" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H83" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I83" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J83" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -2079,6 +3075,18 @@
       <c r="F84">
         <v>330</v>
       </c>
+      <c r="G84" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H84" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I84" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J84" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -2099,6 +3107,18 @@
       <c r="F85">
         <v>210</v>
       </c>
+      <c r="G85" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H85" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I85" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J85" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -2119,6 +3139,18 @@
       <c r="F86">
         <v>48</v>
       </c>
+      <c r="G86" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H86" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I86" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J86" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -2139,6 +3171,18 @@
       <c r="F87">
         <v>48</v>
       </c>
+      <c r="G87" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H87" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I87" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J87" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -2159,6 +3203,18 @@
       <c r="F88">
         <v>48</v>
       </c>
+      <c r="G88" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H88" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I88" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J88" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -2179,6 +3235,18 @@
       <c r="F89">
         <v>88</v>
       </c>
+      <c r="G89" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H89" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I89" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J89" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -2199,6 +3267,18 @@
       <c r="F90">
         <v>110</v>
       </c>
+      <c r="G90" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H90" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I90" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J90" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -2219,6 +3299,18 @@
       <c r="F91">
         <v>110</v>
       </c>
+      <c r="G91" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H91" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I91" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J91" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -2239,6 +3331,18 @@
       <c r="F92">
         <v>912</v>
       </c>
+      <c r="G92" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H92" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I92" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J92" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -2259,6 +3363,18 @@
       <c r="F93">
         <v>110</v>
       </c>
+      <c r="G93" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H93" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I93" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J93" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -2279,6 +3395,18 @@
       <c r="F94">
         <v>96</v>
       </c>
+      <c r="G94" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H94" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I94" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J94" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -2299,6 +3427,18 @@
       <c r="F95">
         <v>330</v>
       </c>
+      <c r="G95" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H95" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I95" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J95" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -2319,6 +3459,18 @@
       <c r="F96">
         <v>210</v>
       </c>
+      <c r="G96" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H96" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I96" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J96" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -2339,6 +3491,18 @@
       <c r="F97">
         <v>48</v>
       </c>
+      <c r="G97" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H97" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I97" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J97" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -2359,6 +3523,18 @@
       <c r="F98">
         <v>96</v>
       </c>
+      <c r="G98" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H98" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I98" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J98" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -2379,6 +3555,18 @@
       <c r="F99">
         <v>48</v>
       </c>
+      <c r="G99" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H99" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I99" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J99" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -2399,6 +3587,18 @@
       <c r="F100">
         <v>48</v>
       </c>
+      <c r="G100" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H100" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I100" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J100" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -2419,6 +3619,18 @@
       <c r="F101">
         <v>912</v>
       </c>
+      <c r="G101" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H101" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I101" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J101" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -2439,6 +3651,18 @@
       <c r="F102">
         <v>96</v>
       </c>
+      <c r="G102" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H102" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I102" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J102" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -2459,6 +3683,18 @@
       <c r="F103">
         <v>330</v>
       </c>
+      <c r="G103" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H103" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I103" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J103" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -2479,6 +3715,18 @@
       <c r="F104">
         <v>210</v>
       </c>
+      <c r="G104" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H104" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I104" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J104" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -2499,6 +3747,18 @@
       <c r="F105">
         <v>110</v>
       </c>
+      <c r="G105" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H105" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I105" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J105" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -2519,6 +3779,18 @@
       <c r="F106">
         <v>48</v>
       </c>
+      <c r="G106" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H106" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I106" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J106" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -2539,6 +3811,18 @@
       <c r="F107">
         <v>144</v>
       </c>
+      <c r="G107" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H107" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I107" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J107" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -2559,6 +3843,18 @@
       <c r="F108">
         <v>912</v>
       </c>
+      <c r="G108" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H108" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I108" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J108" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -2579,6 +3875,18 @@
       <c r="F109">
         <v>96</v>
       </c>
+      <c r="G109" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H109" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I109" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J109" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -2599,6 +3907,18 @@
       <c r="F110">
         <v>330</v>
       </c>
+      <c r="G110" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H110" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I110" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J110" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -2619,6 +3939,18 @@
       <c r="F111">
         <v>210</v>
       </c>
+      <c r="G111" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H111" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I111" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J111" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -2639,6 +3971,18 @@
       <c r="F112">
         <v>110</v>
       </c>
+      <c r="G112" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H112" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I112" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J112" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -2659,6 +4003,18 @@
       <c r="F113">
         <v>48</v>
       </c>
+      <c r="G113" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H113" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I113" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J113" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -2679,6 +4035,18 @@
       <c r="F114">
         <v>48</v>
       </c>
+      <c r="G114" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H114" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I114" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J114" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -2699,6 +4067,18 @@
       <c r="F115">
         <v>144</v>
       </c>
+      <c r="G115" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H115" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I115" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J115" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -2719,6 +4099,18 @@
       <c r="F116">
         <v>1140</v>
       </c>
+      <c r="G116" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H116" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I116" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J116" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -2739,6 +4131,18 @@
       <c r="F117">
         <v>2736</v>
       </c>
+      <c r="G117" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H117" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I117" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J117" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -2759,6 +4163,18 @@
       <c r="F118">
         <v>96</v>
       </c>
+      <c r="G118" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H118" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I118" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J118" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -2779,6 +4195,18 @@
       <c r="F119">
         <v>88</v>
       </c>
+      <c r="G119" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H119" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I119" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J119" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -2799,6 +4227,18 @@
       <c r="F120">
         <v>110</v>
       </c>
+      <c r="G120" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H120" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I120" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J120" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -2819,6 +4259,18 @@
       <c r="F121">
         <v>110</v>
       </c>
+      <c r="G121" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H121" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I121" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J121" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -2839,6 +4291,18 @@
       <c r="F122">
         <v>715</v>
       </c>
+      <c r="G122" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H122" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I122" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J122" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -2859,6 +4323,18 @@
       <c r="F123">
         <v>410</v>
       </c>
+      <c r="G123" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H123" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I123" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J123" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -2879,6 +4355,18 @@
       <c r="F124">
         <v>410</v>
       </c>
+      <c r="G124" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H124" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I124" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J124" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -2899,6 +4387,18 @@
       <c r="F125">
         <v>155</v>
       </c>
+      <c r="G125" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H125" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I125" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J125" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -2919,6 +4419,18 @@
       <c r="F126">
         <v>775</v>
       </c>
+      <c r="G126" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H126" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I126" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J126" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -2939,6 +4451,18 @@
       <c r="F127">
         <v>730</v>
       </c>
+      <c r="G127" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H127" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I127" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J127" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -2959,10 +4483,22 @@
       <c r="F128">
         <v>595</v>
       </c>
+      <c r="G128" t="str">
+        <v>JPI REALTY, INC. 600 E. LAS COLINAS BLVD. #1800 IRVING, TX 75039</v>
+      </c>
+      <c r="H128" t="str">
+        <v>SAUL REYES</v>
+      </c>
+      <c r="I128" t="str">
+        <v>2206JPI02S</v>
+      </c>
+      <c r="J128" t="str">
+        <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F128"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J128"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
some tests that worked out well
</commit_message>
<xml_diff>
--- a/010-npm_node/2206JPI02S Anna Waters Creek REV 3 Signage.xlsx
+++ b/010-npm_node/2206JPI02S Anna Waters Creek REV 3 Signage.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J128"/>
+  <dimension ref="A1:L128"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -431,6 +431,12 @@
       <c r="J1" t="str">
         <v>9</v>
       </c>
+      <c r="K1" t="str">
+        <v>10</v>
+      </c>
+      <c r="L1" t="str">
+        <v>11</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -463,6 +469,12 @@
       <c r="J2" t="str">
         <v>REVISIONS</v>
       </c>
+      <c r="K2" t="str">
+        <v>PROJECT_NAME</v>
+      </c>
+      <c r="L2" t="str">
+        <v>CONTRACT_FILE</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -495,6 +507,12 @@
       <c r="J3" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K3" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L3" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -527,6 +545,12 @@
       <c r="J4" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K4" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L4" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -559,6 +583,12 @@
       <c r="J5" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K5" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L5" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -591,6 +621,12 @@
       <c r="J6" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K6" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L6" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -623,6 +659,12 @@
       <c r="J7" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K7" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -655,6 +697,12 @@
       <c r="J8" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K8" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L8" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -687,6 +735,12 @@
       <c r="J9" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K9" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -719,6 +773,12 @@
       <c r="J10" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K10" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L10" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -751,6 +811,12 @@
       <c r="J11" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K11" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L11" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -783,6 +849,12 @@
       <c r="J12" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K12" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L12" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -815,6 +887,12 @@
       <c r="J13" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K13" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L13" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -847,6 +925,12 @@
       <c r="J14" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K14" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L14" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -879,6 +963,12 @@
       <c r="J15" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K15" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L15" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -911,6 +1001,12 @@
       <c r="J16" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K16" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L16" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -943,6 +1039,12 @@
       <c r="J17" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K17" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L17" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -975,6 +1077,12 @@
       <c r="J18" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K18" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L18" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1007,6 +1115,12 @@
       <c r="J19" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K19" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L19" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1039,6 +1153,12 @@
       <c r="J20" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K20" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L20" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1071,6 +1191,12 @@
       <c r="J21" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K21" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L21" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1103,6 +1229,12 @@
       <c r="J22" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K22" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L22" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1135,6 +1267,12 @@
       <c r="J23" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K23" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L23" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1167,6 +1305,12 @@
       <c r="J24" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K24" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L24" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1199,6 +1343,12 @@
       <c r="J25" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K25" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L25" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1231,6 +1381,12 @@
       <c r="J26" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K26" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L26" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1263,6 +1419,12 @@
       <c r="J27" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K27" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L27" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1295,6 +1457,12 @@
       <c r="J28" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K28" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L28" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1327,6 +1495,12 @@
       <c r="J29" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K29" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L29" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1359,6 +1533,12 @@
       <c r="J30" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K30" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L30" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1391,6 +1571,12 @@
       <c r="J31" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K31" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L31" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1423,6 +1609,12 @@
       <c r="J32" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K32" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L32" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1455,6 +1647,12 @@
       <c r="J33" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K33" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L33" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1487,6 +1685,12 @@
       <c r="J34" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K34" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L34" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1519,6 +1723,12 @@
       <c r="J35" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K35" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L35" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1551,6 +1761,12 @@
       <c r="J36" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K36" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L36" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1583,6 +1799,12 @@
       <c r="J37" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K37" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L37" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1615,6 +1837,12 @@
       <c r="J38" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K38" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L38" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1647,6 +1875,12 @@
       <c r="J39" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K39" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L39" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1679,6 +1913,12 @@
       <c r="J40" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K40" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L40" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1711,6 +1951,12 @@
       <c r="J41" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K41" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L41" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1743,6 +1989,12 @@
       <c r="J42" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K42" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L42" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1775,6 +2027,12 @@
       <c r="J43" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K43" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L43" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1807,6 +2065,12 @@
       <c r="J44" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K44" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L44" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -1839,6 +2103,12 @@
       <c r="J45" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K45" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L45" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1871,6 +2141,12 @@
       <c r="J46" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K46" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L46" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1903,6 +2179,12 @@
       <c r="J47" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K47" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L47" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1935,6 +2217,12 @@
       <c r="J48" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K48" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L48" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1967,6 +2255,12 @@
       <c r="J49" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K49" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L49" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1999,6 +2293,12 @@
       <c r="J50" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K50" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L50" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2031,6 +2331,12 @@
       <c r="J51" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K51" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L51" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2063,6 +2369,12 @@
       <c r="J52" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K52" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L52" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2095,6 +2407,12 @@
       <c r="J53" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K53" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L53" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2127,6 +2445,12 @@
       <c r="J54" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K54" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L54" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2159,6 +2483,12 @@
       <c r="J55" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K55" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L55" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2191,6 +2521,12 @@
       <c r="J56" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K56" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L56" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2223,6 +2559,12 @@
       <c r="J57" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K57" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L57" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2255,6 +2597,12 @@
       <c r="J58" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K58" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L58" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2287,6 +2635,12 @@
       <c r="J59" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K59" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L59" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2319,6 +2673,12 @@
       <c r="J60" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K60" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L60" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2351,6 +2711,12 @@
       <c r="J61" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K61" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L61" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2383,6 +2749,12 @@
       <c r="J62" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K62" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L62" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2415,6 +2787,12 @@
       <c r="J63" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K63" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L63" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2447,6 +2825,12 @@
       <c r="J64" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K64" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L64" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2479,6 +2863,12 @@
       <c r="J65" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K65" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L65" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2511,6 +2901,12 @@
       <c r="J66" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K66" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L66" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2543,6 +2939,12 @@
       <c r="J67" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K67" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L67" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2575,6 +2977,12 @@
       <c r="J68" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K68" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L68" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2607,6 +3015,12 @@
       <c r="J69" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K69" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L69" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2639,6 +3053,12 @@
       <c r="J70" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K70" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L70" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2671,6 +3091,12 @@
       <c r="J71" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K71" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L71" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2703,6 +3129,12 @@
       <c r="J72" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K72" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L72" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2735,6 +3167,12 @@
       <c r="J73" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K73" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L73" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2767,6 +3205,12 @@
       <c r="J74" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K74" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L74" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2799,6 +3243,12 @@
       <c r="J75" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K75" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L75" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2831,6 +3281,12 @@
       <c r="J76" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K76" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L76" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2863,6 +3319,12 @@
       <c r="J77" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K77" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L77" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2895,6 +3357,12 @@
       <c r="J78" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K78" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L78" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2927,6 +3395,12 @@
       <c r="J79" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K79" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L79" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2959,6 +3433,12 @@
       <c r="J80" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K80" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L80" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -2991,6 +3471,12 @@
       <c r="J81" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K81" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L81" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -3023,6 +3509,12 @@
       <c r="J82" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K82" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L82" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -3055,6 +3547,12 @@
       <c r="J83" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K83" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L83" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -3087,6 +3585,12 @@
       <c r="J84" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K84" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L84" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -3119,6 +3623,12 @@
       <c r="J85" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K85" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L85" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -3151,6 +3661,12 @@
       <c r="J86" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K86" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L86" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -3183,6 +3699,12 @@
       <c r="J87" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K87" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L87" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -3215,6 +3737,12 @@
       <c r="J88" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K88" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L88" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -3247,6 +3775,12 @@
       <c r="J89" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K89" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L89" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3279,6 +3813,12 @@
       <c r="J90" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K90" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L90" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -3311,6 +3851,12 @@
       <c r="J91" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K91" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L91" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -3343,6 +3889,12 @@
       <c r="J92" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K92" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L92" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -3375,6 +3927,12 @@
       <c r="J93" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K93" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L93" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -3407,6 +3965,12 @@
       <c r="J94" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K94" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L94" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -3439,6 +4003,12 @@
       <c r="J95" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K95" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L95" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -3471,6 +4041,12 @@
       <c r="J96" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K96" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L96" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -3503,6 +4079,12 @@
       <c r="J97" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K97" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L97" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -3535,6 +4117,12 @@
       <c r="J98" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K98" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L98" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -3567,6 +4155,12 @@
       <c r="J99" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K99" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L99" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -3599,6 +4193,12 @@
       <c r="J100" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K100" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L100" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -3631,6 +4231,12 @@
       <c r="J101" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K101" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L101" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -3663,6 +4269,12 @@
       <c r="J102" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K102" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L102" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -3695,6 +4307,12 @@
       <c r="J103" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K103" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L103" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -3727,6 +4345,12 @@
       <c r="J104" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K104" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L104" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -3759,6 +4383,12 @@
       <c r="J105" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K105" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L105" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -3791,6 +4421,12 @@
       <c r="J106" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K106" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L106" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -3823,6 +4459,12 @@
       <c r="J107" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K107" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L107" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -3855,6 +4497,12 @@
       <c r="J108" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K108" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L108" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -3887,6 +4535,12 @@
       <c r="J109" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K109" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L109" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -3919,6 +4573,12 @@
       <c r="J110" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K110" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L110" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -3951,6 +4611,12 @@
       <c r="J111" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K111" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L111" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -3983,6 +4649,12 @@
       <c r="J112" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K112" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L112" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -4015,6 +4687,12 @@
       <c r="J113" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K113" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L113" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -4047,6 +4725,12 @@
       <c r="J114" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K114" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L114" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -4079,6 +4763,12 @@
       <c r="J115" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K115" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L115" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -4111,6 +4801,12 @@
       <c r="J116" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K116" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L116" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -4143,6 +4839,12 @@
       <c r="J117" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K117" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L117" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -4175,6 +4877,12 @@
       <c r="J118" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K118" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L118" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -4207,6 +4915,12 @@
       <c r="J119" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K119" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L119" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -4239,6 +4953,12 @@
       <c r="J120" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K120" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L120" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -4271,6 +4991,12 @@
       <c r="J121" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K121" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L121" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -4303,6 +5029,12 @@
       <c r="J122" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K122" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L122" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -4335,6 +5067,12 @@
       <c r="J123" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K123" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L123" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -4367,6 +5105,12 @@
       <c r="J124" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K124" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L124" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -4399,6 +5143,12 @@
       <c r="J125" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K125" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L125" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -4431,6 +5181,12 @@
       <c r="J126" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K126" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L126" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -4463,6 +5219,12 @@
       <c r="J127" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K127" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L127" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -4495,10 +5257,16 @@
       <c r="J128" t="str">
         <v>10.13.22 11.20.23 REV 1 11.29.23 REV 2 4.08.24 Rev 3</v>
       </c>
+      <c r="K128" t="str">
+        <v>ANNA WATERS CREEK</v>
+      </c>
+      <c r="L128" t="str">
+        <v>2206JPI02S Anna Waters Creek REV 3 Signage.xlsx</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J128"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L128"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>